<commit_message>
Content 2026-10-12.1: one question each for care level and home ownership
As stated to the client on 2 October (chatting.md section 18):
- rc2 (care level in the residential section) and f2 (home ownership in the
  funding section) removed; q19_level and q6_owns stay;
- q19_level gains the psychogeriatric level;
- the two residential actions now read q19_level, and home support counts
  like no residential level when deciding to suggest an assessment.

The content spreadsheet in deliverables/ is re-exported; it compiles back to
the same content.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
+++ b/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1710" uniqueCount="777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1682" uniqueCount="770">
   <si>
     <t>Ageing Navigator content spreadsheet</t>
   </si>
@@ -903,6 +903,7 @@
 rest_home = Rest home level
 hospital = Hospital level
 dementia = Dementia care
+psychogeriatric = Psychogeriatric care
 none = No level was identified
 unsure = Not sure</t>
   </si>
@@ -934,20 +935,6 @@
 separated = Separated or divorced
 partnered_independent = Married or partnered, partner lives independently
 partnered_both_care = Married or partnered, both have significant care needs
-other = Other
-unsure = Not sure
-prefer_not_to_say = Prefer not to say</t>
-  </si>
-  <si>
-    <t>f2</t>
-  </si>
-  <si>
-    <t>Do they own a home, or have an interest in a home?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes = Yes
-no = No
-village = They live in a retirement village
 other = Other
 unsure = Not sure
 prefer_not_to_say = Prefer not to say</t>
@@ -1194,24 +1181,6 @@
 actively_looking = We're actively looking for somewhere
 urgent = A place may be needed urgently
 unsure = Not sure</t>
-  </si>
-  <si>
-    <t>rc2</t>
-  </si>
-  <si>
-    <t>If a formal assessment has identified a level of care, what level was identified?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rest_home = Rest-home level
-hospital = Hospital level
-dementia = Dementia care
-psychogeriatric = Psychogeriatric care
-other = Another level
-none = No formal level has been identified
-unsure = Not sure</t>
-  </si>
-  <si>
-    <t>q19 in completed, receiving, reassessment or rc1 is assessment_identified</t>
   </si>
   <si>
     <t>rc3</t>
@@ -2264,7 +2233,7 @@
     <t>residential-assessment</t>
   </si>
   <si>
-    <t>(q23 is residential_care or trigger has considering_residential or q8 has residential_care or q6 is residential_care) and (rc2 not answered or rc2 in none, unsure, other)</t>
+    <t>(q23 is residential_care or trigger has considering_residential or q8 has residential_care or q6 is residential_care) and (q19_level not answered or q19_level in none, unsure, home_support)</t>
   </si>
   <si>
     <t>Ask how an assessment for residential care is arranged</t>
@@ -2288,7 +2257,7 @@
     <t>residential-search</t>
   </si>
   <si>
-    <t>rc1 in assessment_identified, actively_looking, urgent and rc2 in rest_home, hospital, dementia, psychogeriatric</t>
+    <t>rc1 in assessment_identified, actively_looking, urgent and q19_level in rest_home, hospital, dementia, psychogeriatric</t>
   </si>
   <si>
     <t>Shortlist care homes that provide the assessed level of care</t>
@@ -3456,7 +3425,7 @@
         <v>47</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>711</v>
+        <v>704</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>94</v>
@@ -3464,21 +3433,21 @@
     </row>
     <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>712</v>
+        <v>705</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>713</v>
+        <v>706</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>714</v>
+        <v>707</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>715</v>
+        <v>708</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>79</v>
@@ -3486,10 +3455,10 @@
     </row>
     <row r="4" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>717</v>
+        <v>710</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>83</v>
@@ -3497,10 +3466,10 @@
     </row>
     <row r="5" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>718</v>
+        <v>711</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>719</v>
+        <v>712</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>1</v>
@@ -3532,336 +3501,336 @@
         <v>48</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>720</v>
+        <v>713</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>721</v>
+        <v>714</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>722</v>
+        <v>715</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>723</v>
+        <v>716</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>724</v>
+        <v>717</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>725</v>
+        <v>718</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>641</v>
+        <v>634</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>727</v>
+        <v>720</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>728</v>
+        <v>721</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>729</v>
+        <v>722</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>730</v>
+        <v>723</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>731</v>
+        <v>724</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>616</v>
+        <v>609</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>732</v>
+        <v>725</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>612</v>
+        <v>605</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>733</v>
+        <v>726</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>734</v>
+        <v>727</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>612</v>
+        <v>605</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>736</v>
+        <v>729</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>597</v>
+        <v>590</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>737</v>
+        <v>730</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>727</v>
+        <v>720</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>738</v>
+        <v>731</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>535</v>
+        <v>528</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>739</v>
+        <v>732</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>740</v>
+        <v>733</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>741</v>
+        <v>734</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>742</v>
+        <v>735</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>743</v>
+        <v>736</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>740</v>
+        <v>733</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>744</v>
+        <v>737</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>745</v>
+        <v>738</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>746</v>
+        <v>739</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>724</v>
+        <v>717</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>747</v>
+        <v>740</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>549</v>
+        <v>542</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>748</v>
+        <v>741</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>727</v>
+        <v>720</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>749</v>
+        <v>742</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>750</v>
+        <v>743</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>751</v>
+        <v>744</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>752</v>
+        <v>745</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>753</v>
+        <v>746</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>754</v>
+        <v>747</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>755</v>
+        <v>748</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>756</v>
+        <v>749</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>757</v>
+        <v>750</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>759</v>
+        <v>752</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>759</v>
+        <v>752</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>760</v>
+        <v>753</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>761</v>
+        <v>754</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>762</v>
+        <v>755</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>763</v>
+        <v>756</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>768</v>
+        <v>761</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>769</v>
+        <v>762</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>770</v>
+        <v>763</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>771</v>
+        <v>764</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>772</v>
+        <v>765</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>455</v>
+        <v>448</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>774</v>
+        <v>767</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>775</v>
+        <v>768</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
     </row>
   </sheetData>
@@ -5735,10 +5704,10 @@
         <v>225</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>1</v>
+        <v>226</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>1</v>
@@ -5764,7 +5733,7 @@
     </row>
     <row r="37" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>71</v>
@@ -5776,10 +5745,10 @@
         <v>111</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>229</v>
+        <v>1</v>
       </c>
       <c r="G37" s="4" t="s">
         <v>230</v>
@@ -5811,22 +5780,22 @@
         <v>231</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>111</v>
+        <v>232</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>1</v>
+        <v>234</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>1</v>
@@ -5841,7 +5810,7 @@
         <v>1</v>
       </c>
       <c r="L38" s="4" t="s">
-        <v>1</v>
+        <v>236</v>
       </c>
       <c r="M38" s="4" t="s">
         <v>1</v>
@@ -5852,7 +5821,7 @@
     </row>
     <row r="39" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>75</v>
@@ -5861,16 +5830,16 @@
         <v>1</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>235</v>
+        <v>111</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>237</v>
+        <v>1</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H39" s="4" t="s">
         <v>1</v>
@@ -5885,7 +5854,7 @@
         <v>1</v>
       </c>
       <c r="L39" s="4" t="s">
-        <v>239</v>
+        <v>1</v>
       </c>
       <c r="M39" s="4" t="s">
         <v>1</v>
@@ -5899,7 +5868,7 @@
         <v>240</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>1</v>
@@ -5949,19 +5918,19 @@
         <v>1</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>244</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="G41" s="4" t="s">
         <v>245</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>1</v>
+        <v>246</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>1</v>
@@ -5984,28 +5953,28 @@
     </row>
     <row r="42" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>1</v>
+        <v>79</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>139</v>
+        <v>1</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>249</v>
+        <v>1</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>1</v>
@@ -6037,7 +6006,7 @@
         <v>79</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>251</v>
@@ -6046,7 +6015,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>252</v>
+        <v>1</v>
       </c>
       <c r="H43" s="4" t="s">
         <v>1</v>
@@ -6064,7 +6033,7 @@
         <v>1</v>
       </c>
       <c r="M43" s="4" t="s">
-        <v>1</v>
+        <v>252</v>
       </c>
       <c r="N43" s="4" t="s">
         <v>1</v>
@@ -6081,16 +6050,16 @@
         <v>79</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>125</v>
+        <v>104</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>254</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>1</v>
+        <v>255</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>1</v>
@@ -6108,7 +6077,7 @@
         <v>1</v>
       </c>
       <c r="M44" s="4" t="s">
-        <v>255</v>
+        <v>1</v>
       </c>
       <c r="N44" s="4" t="s">
         <v>1</v>
@@ -6125,13 +6094,13 @@
         <v>79</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>257</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>139</v>
+        <v>1</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>258</v>
@@ -6213,19 +6182,19 @@
         <v>79</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>263</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="G47" s="4" t="s">
         <v>264</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>1</v>
@@ -6257,19 +6226,19 @@
         <v>79</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>266</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>139</v>
+        <v>1</v>
       </c>
       <c r="G48" s="4" t="s">
         <v>267</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>1</v>
@@ -6339,22 +6308,22 @@
         <v>271</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>111</v>
       </c>
       <c r="E50" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G50" s="4" t="s">
         <v>272</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>273</v>
       </c>
       <c r="H50" s="4" t="s">
         <v>1</v>
@@ -6380,7 +6349,7 @@
     </row>
     <row r="51" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>83</v>
@@ -6389,19 +6358,19 @@
         <v>83</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>158</v>
+        <v>274</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="G51" s="4" t="s">
         <v>275</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>1</v>
@@ -6427,10 +6396,10 @@
         <v>276</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>111</v>
@@ -6460,7 +6429,7 @@
         <v>1</v>
       </c>
       <c r="M52" s="4" t="s">
-        <v>279</v>
+        <v>1</v>
       </c>
       <c r="N52" s="4" t="s">
         <v>1</v>
@@ -6468,28 +6437,28 @@
     </row>
     <row r="53" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E53" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="B53" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="E53" s="4" t="s">
+      <c r="F53" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G53" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="F53" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>282</v>
-      </c>
       <c r="H53" s="4" t="s">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>1</v>
@@ -6512,7 +6481,7 @@
     </row>
     <row r="54" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>87</v>
@@ -6524,19 +6493,19 @@
         <v>111</v>
       </c>
       <c r="E54" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G54" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="F54" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>285</v>
-      </c>
       <c r="H54" s="4" t="s">
         <v>1</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>1</v>
+        <v>210</v>
       </c>
       <c r="J54" s="4" t="s">
         <v>109</v>
@@ -6556,7 +6525,7 @@
     </row>
     <row r="55" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>87</v>
@@ -6568,10 +6537,10 @@
         <v>111</v>
       </c>
       <c r="E55" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="F55" s="4" t="s">
         <v>287</v>
-      </c>
-      <c r="F55" s="4" t="s">
-        <v>1</v>
       </c>
       <c r="G55" s="4" t="s">
         <v>288</v>
@@ -6603,28 +6572,28 @@
         <v>289</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>290</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="G56" s="4" t="s">
         <v>291</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>1</v>
+        <v>292</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>210</v>
+        <v>1</v>
       </c>
       <c r="J56" s="4" t="s">
         <v>109</v>
@@ -6644,25 +6613,25 @@
     </row>
     <row r="57" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>295</v>
+        <v>1</v>
       </c>
       <c r="H57" s="4" t="s">
         <v>1</v>
@@ -6671,7 +6640,7 @@
         <v>1</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>109</v>
+        <v>150</v>
       </c>
       <c r="K57" s="4" t="s">
         <v>1</v>
@@ -6691,7 +6660,7 @@
         <v>296</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>1</v>
@@ -6712,7 +6681,7 @@
         <v>299</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>1</v>
+        <v>210</v>
       </c>
       <c r="J58" s="4" t="s">
         <v>109</v>
@@ -6735,13 +6704,13 @@
         <v>300</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>147</v>
+        <v>104</v>
       </c>
       <c r="E59" s="4" t="s">
         <v>301</v>
@@ -6750,19 +6719,19 @@
         <v>302</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>1</v>
+        <v>303</v>
       </c>
       <c r="H59" s="4" t="s">
         <v>1</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>1</v>
+        <v>210</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>150</v>
+        <v>109</v>
       </c>
       <c r="K59" s="4" t="s">
-        <v>1</v>
+        <v>304</v>
       </c>
       <c r="L59" s="4" t="s">
         <v>1</v>
@@ -6776,7 +6745,7 @@
     </row>
     <row r="60" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>91</v>
@@ -6785,25 +6754,25 @@
         <v>1</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>104</v>
+        <v>147</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>139</v>
+        <v>1</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>305</v>
+        <v>1</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>306</v>
+        <v>1</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>210</v>
+        <v>1</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>109</v>
+        <v>150</v>
       </c>
       <c r="K60" s="4" t="s">
         <v>1</v>
@@ -6818,94 +6787,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="E61" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="F61" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="H61" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I61" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="J61" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="K61" s="4" t="s">
-        <v>311</v>
-      </c>
-      <c r="L61" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="M61" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="N61" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E62" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="F62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="H62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J62" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="K62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="M62" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="N62" s="4" t="s">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="61" spans="4:10" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="4:10" x14ac:dyDescent="0.25"/>
     <row r="63" spans="4:10" x14ac:dyDescent="0.25"/>
     <row r="64" spans="4:10" x14ac:dyDescent="0.25"/>
     <row r="65" spans="4:10" x14ac:dyDescent="0.25"/>
@@ -7080,50 +6963,50 @@
         <v>47</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>324</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -7131,16 +7014,16 @@
         <v>79</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -7151,13 +7034,13 @@
         <v>84</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -7168,13 +7051,13 @@
         <v>84</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="5:5" x14ac:dyDescent="0.25"/>
@@ -7407,282 +7290,282 @@
         <v>50</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>334</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>341</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>373</v>
-      </c>
       <c r="D15" s="4" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" spans="5:5" x14ac:dyDescent="0.25"/>
@@ -7903,278 +7786,278 @@
         <v>41</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>50</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>384</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>385</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>390</v>
-      </c>
       <c r="M1" s="3" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>44</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="L2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>163</v>
       </c>
       <c r="E3" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>402</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>405</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>407</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>408</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>409</v>
-      </c>
       <c r="M3" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>411</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>412</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>418</v>
-      </c>
       <c r="L4" s="4" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>419</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>420</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>423</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>425</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>426</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>427</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>428</v>
-      </c>
       <c r="L5" s="4" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>436</v>
-      </c>
       <c r="L6" s="4" t="s">
         <v>1</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>440</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>443</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>444</v>
-      </c>
       <c r="K7" s="4" t="s">
         <v>1</v>
       </c>
@@ -8182,163 +8065,163 @@
         <v>1</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>445</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="J8" s="4" t="s">
         <v>446</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>447</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="L8" s="4" t="s">
         <v>448</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>449</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>450</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>451</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>452</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>453</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>454</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>455</v>
-      </c>
       <c r="M8" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="J9" s="4" t="s">
         <v>457</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="K9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L9" s="4" t="s">
         <v>458</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>459</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>460</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>461</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>462</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>464</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>465</v>
-      </c>
       <c r="M9" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J10" s="4" t="s">
         <v>466</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="K10" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>469</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>470</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>471</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>472</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>474</v>
-      </c>
       <c r="L10" s="4" t="s">
         <v>1</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="J11" s="4" t="s">
         <v>475</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>476</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>478</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>479</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>480</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>481</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>482</v>
-      </c>
       <c r="K11" s="4" t="s">
         <v>1</v>
       </c>
@@ -8346,121 +8229,121 @@
         <v>1</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="I12" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="J12" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="K12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L12" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>486</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>487</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>488</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>489</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>490</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>491</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>492</v>
-      </c>
       <c r="M12" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="13" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>1</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>1</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>1</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>1</v>
@@ -8469,197 +8352,197 @@
         <v>1</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J15" s="4" t="s">
         <v>507</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="K15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L15" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>509</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>510</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>511</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>512</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>513</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>515</v>
-      </c>
       <c r="M15" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="16" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="K16" s="4" t="s">
         <v>516</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="L16" s="4" t="s">
         <v>517</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>518</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>519</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>520</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>521</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>522</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="L16" s="4" t="s">
-        <v>524</v>
-      </c>
       <c r="M16" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>525</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="J17" s="4" t="s">
         <v>526</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="K17" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="L17" s="4" t="s">
         <v>528</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>529</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>530</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>531</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>532</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>533</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>534</v>
-      </c>
-      <c r="L17" s="4" t="s">
-        <v>535</v>
-      </c>
       <c r="M17" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="s">
         <v>536</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>526</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>537</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>538</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>539</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>540</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>541</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>542</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>543</v>
-      </c>
       <c r="L18" s="4" t="s">
         <v>1</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>544</v>
+        <v>537</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>545</v>
+        <v>538</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>546</v>
+        <v>539</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>547</v>
+        <v>540</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>548</v>
+        <v>541</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>1</v>
@@ -8671,36 +8554,36 @@
         <v>1</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>549</v>
+        <v>542</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="20" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>551</v>
+        <v>544</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>1</v>
@@ -8712,323 +8595,323 @@
         <v>1</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="21" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L21" s="4" t="s">
         <v>557</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>558</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>537</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>559</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>560</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>561</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>562</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>563</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L21" s="4" t="s">
-        <v>564</v>
-      </c>
       <c r="M21" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="22" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="I22" s="4" t="s">
         <v>565</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="J22" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="K22" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>568</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>569</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>570</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>571</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>572</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>573</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>574</v>
-      </c>
       <c r="L22" s="4" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="23" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
+        <v>568</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="K23" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="E23" s="4" t="s">
+      <c r="L23" s="4" t="s">
         <v>576</v>
       </c>
-      <c r="F23" s="4" t="s">
-        <v>577</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>578</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>579</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>580</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>581</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>582</v>
-      </c>
-      <c r="L23" s="4" t="s">
-        <v>583</v>
-      </c>
       <c r="M23" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="24" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>587</v>
+        <v>580</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>588</v>
+        <v>581</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>1</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>589</v>
+        <v>582</v>
       </c>
       <c r="K24" s="4" t="s">
         <v>1</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="M24" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="25" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>591</v>
+        <v>584</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>593</v>
+        <v>586</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>594</v>
+        <v>587</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>1</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>595</v>
+        <v>588</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>596</v>
+        <v>589</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>597</v>
+        <v>590</v>
       </c>
       <c r="M25" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>598</v>
+        <v>591</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D26" s="4" t="s">
+        <v>592</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="K26" s="4" t="s">
         <v>599</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>600</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>601</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>602</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>603</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>604</v>
-      </c>
-      <c r="J26" s="4" t="s">
-        <v>605</v>
-      </c>
-      <c r="K26" s="4" t="s">
-        <v>606</v>
-      </c>
       <c r="L26" s="4" t="s">
-        <v>455</v>
+        <v>448</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="27" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>607</v>
+        <v>600</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D27" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>602</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>604</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="K27" s="4" t="s">
         <v>608</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="L27" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="F27" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>611</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>612</v>
-      </c>
-      <c r="I27" s="4" t="s">
-        <v>613</v>
-      </c>
-      <c r="J27" s="4" t="s">
-        <v>614</v>
-      </c>
-      <c r="K27" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="L27" s="4" t="s">
-        <v>616</v>
-      </c>
       <c r="M27" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="28" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>618</v>
+        <v>611</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>619</v>
+        <v>612</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>620</v>
+        <v>613</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>621</v>
+        <v>614</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>622</v>
+        <v>615</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>623</v>
+        <v>616</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>1</v>
@@ -9043,33 +8926,33 @@
         <v>1</v>
       </c>
       <c r="M28" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="29" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>624</v>
+        <v>617</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>625</v>
+        <v>618</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>626</v>
+        <v>619</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>627</v>
+        <v>620</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>628</v>
+        <v>621</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>629</v>
+        <v>622</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>618</v>
+        <v>611</v>
       </c>
       <c r="I29" s="4" t="s">
         <v>1</v>
@@ -9084,7 +8967,7 @@
         <v>1</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.25"/>
@@ -9304,197 +9187,197 @@
         <v>48</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>630</v>
+        <v>623</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>631</v>
+        <v>624</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>632</v>
+        <v>625</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>633</v>
+        <v>626</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>634</v>
+        <v>627</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>635</v>
+        <v>628</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>631</v>
+        <v>624</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>636</v>
+        <v>629</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>637</v>
+        <v>630</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>616</v>
+        <v>609</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>638</v>
+        <v>631</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>631</v>
+        <v>624</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>640</v>
+        <v>633</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>641</v>
+        <v>634</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>643</v>
+        <v>636</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>644</v>
+        <v>637</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>645</v>
+        <v>638</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>646</v>
+        <v>639</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>647</v>
+        <v>640</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>648</v>
+        <v>641</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>649</v>
+        <v>642</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>651</v>
+        <v>644</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>1</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>652</v>
+        <v>645</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>648</v>
+        <v>641</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>653</v>
+        <v>646</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>654</v>
+        <v>647</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>597</v>
+        <v>590</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>655</v>
+        <v>648</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>648</v>
+        <v>641</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>656</v>
+        <v>649</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>657</v>
+        <v>650</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>648</v>
+        <v>641</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>658</v>
+        <v>651</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>659</v>
+        <v>652</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>660</v>
+        <v>653</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>1</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="7:7" x14ac:dyDescent="0.25"/>
@@ -9716,207 +9599,207 @@
         <v>41</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>662</v>
+        <v>655</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>664</v>
+        <v>657</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>666</v>
+        <v>659</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>667</v>
+        <v>660</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>668</v>
+        <v>661</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>669</v>
+        <v>662</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>670</v>
+        <v>663</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>671</v>
+        <v>664</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>672</v>
+        <v>665</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>673</v>
+        <v>666</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>674</v>
+        <v>667</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>675</v>
+        <v>668</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>676</v>
+        <v>669</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>677</v>
+        <v>670</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>678</v>
+        <v>671</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>680</v>
+        <v>673</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>682</v>
+        <v>675</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>683</v>
+        <v>676</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>684</v>
+        <v>677</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>687</v>
+        <v>680</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>688</v>
+        <v>681</v>
       </c>
     </row>
     <row r="16" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>689</v>
+        <v>682</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>692</v>
+        <v>685</v>
       </c>
     </row>
     <row r="18" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>693</v>
+        <v>686</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>694</v>
+        <v>687</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>696</v>
+        <v>689</v>
       </c>
     </row>
     <row r="20" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>697</v>
+        <v>690</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>698</v>
+        <v>691</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>699</v>
+        <v>692</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
     </row>
     <row r="22" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
     </row>
     <row r="23" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>703</v>
+        <v>696</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>704</v>
+        <v>697</v>
       </c>
     </row>
     <row r="24" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>705</v>
+        <v>698</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>706</v>
+        <v>699</v>
       </c>
     </row>
     <row r="25" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>707</v>
+        <v>700</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>708</v>
+        <v>701</v>
       </c>
     </row>
     <row r="26" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>709</v>
+        <v>702</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
His notes of 15 October: old card links work, his opening page text, much bigger text
- The older card links on his site (respite, planning_ahead; also not_sure,
  support_needs) are accepted as aliases, so they pre-select their card.
- Opening page in his words: shorter test banner, his intro, a "Before you
  start" heading, his consent and news wording, his line under Start; a
  privacy_policy_url text adds "Read our Privacy Policy" once he has a page.
  Content 2026-10-15.2.
- Family pages much larger (like myagedcare.gov.au, as he asked): body 20 px,
  larger headings, cards and controls; no small print; the card-screen note
  removed. Navigator screens unchanged.
- 105 tests, browser check clean (axe, keyboard, desktop, 390 px), no
  sideways scroll at 320 px.
- chatting.md section 35: one message for his notes and the care home list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
+++ b/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
@@ -2482,13 +2482,13 @@
     <t>consent</t>
   </si>
   <si>
-    <t>Ageing Navigator will use your answers to prepare a personalised Family Ageing Action Plan, which you receive as soon as you finish. Your answers are stored securely in Australia, seen only by the Ageing Navigator team, and deleted 12 months after your plan is sent, or sooner if you ask. We do not use AI, and we do not share your answers with anyone else without asking you first.</t>
+    <t>Your information is stored securely in Australia, kept for up to 12 months, and won’t be shared with other organisations without your permission.</t>
   </si>
   <si>
     <t>consent_checkbox</t>
   </si>
   <si>
-    <t>I agree, and I have the older person's agreement or am acting in their interests.</t>
+    <t>I agree, and I have the older person’s agreement or am acting in their interests.</t>
   </si>
   <si>
     <t>thank_you</t>
@@ -2570,7 +2570,7 @@
     <t>marketing_consent</t>
   </si>
   <si>
-    <t>Send me occasional news from Ageing Navigator. This is optional and you can stop at any time.</t>
+    <t>Send me occasional Ageing Navigator news. Optional.</t>
   </si>
   <si>
     <t>cta_stay_home</t>
@@ -2606,10 +2606,9 @@
     <t>questionnaire_intro</t>
   </si>
   <si>
-    <t xml:space="preserve">Tell us what's happening, and we'll help you work out what to do next.
-This questionnaire prepares your free personalised Family Ageing Action Plan. Depending on your situation it takes around 10 to 15 minutes, and you will only be shown questions that are relevant to you.
-You don't need to know every answer. “Not sure” is useful information too.
-Please don't include account numbers, passwords, detailed medical records or other highly confidential information.</t>
+    <t xml:space="preserve">Tell us what’s happening and we’ll help you work out what to do next with a free personalised Family Ageing Action Plan.
+It usually takes around 10 minutes, and you’ll only see questions relevant to your situation. It’s fine to choose “Not sure”.
+Please don’t include passwords, account numbers or detailed medical records.</t>
   </si>
   <si>
     <t>contact_intro</t>

</xml_diff>

<commit_message>
Add useful contacts from the client's list of organisations
Every plan now ends with the organisations from his Repository sheet's
Organisations tab that go with its actions, before the Sources.
- npm run contacts:import reads the tab and his Status Guide into
  content/pilot/contacts.json: name, phone, email, website, coverage.
  Rows marked "Review due" or "Superseded" are left out; his notes are
  never imported.
- Each contact is linked to action keys (defaults in the import script,
  or his optional "Show with actions" column); Seniorline is on every
  plan. A contact leaves the plan with its actions.
- Local organisations show only to families in the areas they serve.
- Page, PDF and review box I; tap-to-call numbers on the web page.
- Content 2026-10-15.3 (contacts_intro), spreadsheet re-exported.
- Navigator guide v4 and Handover note v3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
+++ b/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="778">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1690" uniqueCount="780">
   <si>
     <t>Ageing Navigator content spreadsheet</t>
   </si>
@@ -2627,6 +2627,12 @@
   </si>
   <si>
     <t>A needs assessment decides which level of care is needed, so the levels each home offers are shown.</t>
+  </si>
+  <si>
+    <t>contacts_intro</t>
+  </si>
+  <si>
+    <t>These organisations may be able to help with the actions in your plan. Services and contact details can change, so please check with each organisation directly.</t>
   </si>
   <si>
     <t>Label</t>
@@ -3457,7 +3463,7 @@
         <v>49</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>96</v>
@@ -3465,10 +3471,10 @@
     </row>
     <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>314</v>
@@ -3476,10 +3482,10 @@
     </row>
     <row r="3" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>81</v>
@@ -3487,10 +3493,10 @@
     </row>
     <row r="4" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>85</v>
@@ -3498,10 +3504,10 @@
     </row>
     <row r="5" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>1</v>
@@ -3533,13 +3539,13 @@
         <v>50</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3547,16 +3553,16 @@
         <v>406</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3567,13 +3573,13 @@
         <v>636</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>731</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>729</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3581,16 +3587,16 @@
         <v>521</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3598,33 +3604,33 @@
         <v>613</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>609</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>609</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3632,16 +3638,16 @@
         <v>594</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3649,50 +3655,50 @@
         <v>532</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>745</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>746</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>743</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>744</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>741</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3700,16 +3706,16 @@
         <v>546</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3717,16 +3723,16 @@
         <v>462</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3734,16 +3740,16 @@
         <v>553</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3751,16 +3757,16 @@
         <v>580</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3768,16 +3774,16 @@
         <v>489</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3785,16 +3791,16 @@
         <v>512</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3802,50 +3808,50 @@
         <v>561</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3853,16 +3859,16 @@
         <v>452</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
   </sheetData>
@@ -9619,7 +9625,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -9850,6 +9856,14 @@
         <v>711</v>
       </c>
     </row>
+    <row r="29" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>712</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>713</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Add the privacy policy page, as a draft for the client's approval
- /privacy shows content/pilot/privacy-policy.md (front matter: updated,
  status). While it is a draft, the page says it awaits approval.
- The consent's "Read our Privacy Policy." now links to it (content
  2026-10-15.4, privacy_policy_url), and every family page's footer too.
- The wording follows how the pilot works: what is collected and why,
  who sees it, Supabase (Sydney), Vercel and Resend, no AI, browser
  storage, 12 months' retention, access, correction and deletion, the
  Privacy Commissioner. tests/privacy.test.ts checks it against the
  app's settings.
- doc:pdf reads front matter and takes an output path; review copy in
  deliverables/Privacy-policy-draft.pdf. marked is now a dependency.
- The expired-link page no longer prints an empty phone number.
- Privacy facts v3; Handover note and Navigator guide updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
+++ b/deliverables/Ageing-Navigator-content-spreadsheet.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1690" uniqueCount="780">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="782">
   <si>
     <t>Ageing Navigator content spreadsheet</t>
   </si>
@@ -2627,6 +2627,12 @@
   </si>
   <si>
     <t>A needs assessment decides which level of care is needed, so the levels each home offers are shown.</t>
+  </si>
+  <si>
+    <t>privacy_policy_url</t>
+  </si>
+  <si>
+    <t>/privacy</t>
   </si>
   <si>
     <t>contacts_intro</t>
@@ -3463,7 +3469,7 @@
         <v>49</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>96</v>
@@ -3471,10 +3477,10 @@
     </row>
     <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>314</v>
@@ -3482,10 +3488,10 @@
     </row>
     <row r="3" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>81</v>
@@ -3493,10 +3499,10 @@
     </row>
     <row r="4" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>85</v>
@@ -3504,10 +3510,10 @@
     </row>
     <row r="5" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>1</v>
@@ -3539,13 +3545,13 @@
         <v>50</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3553,16 +3559,16 @@
         <v>406</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3573,13 +3579,13 @@
         <v>636</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>733</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>731</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3587,16 +3593,16 @@
         <v>521</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3604,33 +3610,33 @@
         <v>613</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>609</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>609</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3638,16 +3644,16 @@
         <v>594</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3655,50 +3661,50 @@
         <v>532</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>747</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>748</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>745</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>746</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>743</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3706,16 +3712,16 @@
         <v>546</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3723,16 +3729,16 @@
         <v>462</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3740,16 +3746,16 @@
         <v>553</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3757,16 +3763,16 @@
         <v>580</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3774,16 +3780,16 @@
         <v>489</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3791,16 +3797,16 @@
         <v>512</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3808,50 +3814,50 @@
         <v>561</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -3859,16 +3865,16 @@
         <v>452</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
   </sheetData>
@@ -9625,7 +9631,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -9864,6 +9870,14 @@
         <v>713</v>
       </c>
     </row>
+    <row r="30" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>714</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>715</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>